<commit_message>
ciclo de vendas koru
</commit_message>
<xml_diff>
--- a/public/data/Funil Vendas Externas.xlsx
+++ b/public/data/Funil Vendas Externas.xlsx
@@ -14,7 +14,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -40,8 +45,13 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle builtinId="0" name="Normal" xfId="0"/>
@@ -52,7 +62,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetData>
-    <row r="1" spans="1:44">
+    <row r="1" spans="1:45">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>ID</t>
@@ -250,244 +260,464 @@
       </c>
       <c r="AN1" s="0" t="inlineStr">
         <is>
+          <t>Termos do usuário (contato)</t>
+        </is>
+      </c>
+      <c r="AO1" s="0" t="inlineStr">
+        <is>
           <t>Nota 1</t>
         </is>
       </c>
-      <c r="AO1" s="0" t="inlineStr">
+      <c r="AP1" s="0" t="inlineStr">
         <is>
           <t>Nota 2</t>
         </is>
       </c>
-      <c r="AP1" s="0" t="inlineStr">
+      <c r="AQ1" s="0" t="inlineStr">
         <is>
           <t>Nota 3</t>
         </is>
       </c>
-      <c r="AQ1" s="0" t="inlineStr">
+      <c r="AR1" s="0" t="inlineStr">
         <is>
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="AR1" s="0" t="inlineStr">
+      <c r="AS1" s="0" t="inlineStr">
         <is>
           <t>Nota 5</t>
         </is>
       </c>
     </row>
-    <row r="2" spans="1:39">
+    <row r="2" spans="1:41">
       <c r="A2" s="0">
+        <v>36987424</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>JOSE DEUSDETE</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>Negociação</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>Funil Vendas Externas</t>
+        </is>
+      </c>
+      <c r="I2" s="0">
+        <v>245000000</v>
+      </c>
+      <c r="J2" s="0" t="inlineStr">
+        <is>
+          <t>16.04.2026 08:13:28</t>
+        </is>
+      </c>
+      <c r="K2" s="0" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L2" s="0" t="inlineStr">
+        <is>
+          <t>16.04.2026 08:16:40</t>
+        </is>
+      </c>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="N2" s="0" t="inlineStr">
+        <is>
+          <t>Eduardo Martins</t>
+        </is>
+      </c>
+      <c r="P2" s="0" t="inlineStr">
+        <is>
+          <t>não fechado</t>
+        </is>
+      </c>
+      <c r="R2" s="0" t="inlineStr">
+        <is>
+          <t>Alameda dos ipês</t>
+        </is>
+      </c>
+      <c r="S2" s="0" t="inlineStr">
+        <is>
+          <t>Imobiliária</t>
+        </is>
+      </c>
+      <c r="AO2" s="0" t="inlineStr">
+        <is>
+          <t>Cliente aprovado:
+Aguardando corretor agendar visita no stand com o cliente para montar o fluxo de pagamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:41">
+      <c r="A3" s="1">
+        <v>36968686</v>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>FRANCISCO VALTER</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Negociação</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Funil Vendas Externas</t>
+        </is>
+      </c>
+      <c r="I3" s="1">
+        <v>245000000</v>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>15.04.2026 17:18:37</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>16.04.2026 08:12:31</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>não fechado</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>Alameda dos ipês</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>Imobiliária</t>
+        </is>
+      </c>
+      <c r="AO3" s="1" t="inlineStr">
+        <is>
+          <t>Cliente condicionado. 
+Nova proposta: 
+Corretor que seguir com o contrato apenas com a simulação, recebendo o sinal de R$ 5.000,00 e tentando outra avaliação daqui a 3 meses, junto com a resposta do moradia Ceará.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:41">
+      <c r="A4" s="1">
+        <v>36965162</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>KELSON DA SILVA</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Analise de credito</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Funil Vendas Externas</t>
+        </is>
+      </c>
+      <c r="I4" s="1">
+        <v>245000000</v>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>15.04.2026 15:49:06</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>15.04.2026 16:41:35</t>
+        </is>
+      </c>
+      <c r="M4" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="N4" s="1" t="inlineStr">
+        <is>
+          <t>Jean</t>
+        </is>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>não fechado</t>
+        </is>
+      </c>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>Alameda dos ipês</t>
+        </is>
+      </c>
+      <c r="S4" s="1" t="inlineStr">
+        <is>
+          <t>Imobiliária</t>
+        </is>
+      </c>
+      <c r="AO4" s="1" t="inlineStr">
+        <is>
+          <t>Aguardando retificação do imposto de renda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:41">
+      <c r="A5" s="1">
+        <v>36965090</v>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>JONATAS SANTOS</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Negociação</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>Funil Vendas Externas</t>
+        </is>
+      </c>
+      <c r="I5" s="1">
+        <v>245000000</v>
+      </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>15.04.2026 15:47:08</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>16.04.2026 08:12:36</t>
+        </is>
+      </c>
+      <c r="M5" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="N5" s="1" t="inlineStr">
+        <is>
+          <t>Furtado Oliv. Imóveis, Ilberto</t>
+        </is>
+      </c>
+      <c r="P5" s="1" t="inlineStr">
+        <is>
+          <t>não fechado</t>
+        </is>
+      </c>
+      <c r="R5" s="1" t="inlineStr">
+        <is>
+          <t>Alameda doa ipês</t>
+        </is>
+      </c>
+      <c r="S5" s="1" t="inlineStr">
+        <is>
+          <t>Imobiliária</t>
+        </is>
+      </c>
+      <c r="AO5" s="1" t="inlineStr">
+        <is>
+          <t>Cliente condicionado. 
+Ajustando proposta:
+Corretor gostaria de seguir com a aprovação que temos, colocando dois balões no valor R$ 3.500,00.
+Primeiro para Agosto/2026, segundo para Dezembro/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:40">
+      <c r="A6" s="1">
         <v>36631874</v>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Bianca Katila Oliveira</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t>Analise de credito</t>
-        </is>
-      </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Venda ganha</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>Funil Vendas Externas</t>
         </is>
       </c>
-      <c r="I2" s="0">
+      <c r="I6" s="1">
         <v>242000000</v>
       </c>
-      <c r="J2" s="0" t="inlineStr">
+      <c r="J6" s="1" t="inlineStr">
         <is>
           <t>08.04.2026 10:00:16</t>
         </is>
       </c>
-      <c r="K2" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="L2" s="0" t="inlineStr">
-        <is>
-          <t>08.04.2026 11:11:33</t>
-        </is>
-      </c>
-      <c r="M2" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="N2" s="0" t="inlineStr">
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>09.04.2026 17:18:53</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="N6" s="1" t="inlineStr">
         <is>
           <t>Italo, Cassia Aguiar</t>
         </is>
       </c>
-      <c r="P2" s="0" t="inlineStr">
-        <is>
-          <t>não fechado</t>
-        </is>
-      </c>
-      <c r="R2" s="0" t="inlineStr">
+      <c r="P6" s="1" t="inlineStr">
+        <is>
+          <t>09.04.2026 17:18</t>
+        </is>
+      </c>
+      <c r="R6" s="1" t="inlineStr">
         <is>
           <t>Alameda dos ipês</t>
         </is>
       </c>
-      <c r="S2" s="0" t="inlineStr">
+      <c r="S6" s="1" t="inlineStr">
         <is>
           <t>Imobiliária</t>
         </is>
       </c>
     </row>
-    <row r="3" spans="1:40">
-      <c r="A3" s="0">
-        <v>36240978</v>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>Maria Clara</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
+    <row r="7" spans="1:41">
+      <c r="A7" s="1">
+        <v>36033076</v>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Larissa</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>Comercial</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t>Analise de credito</t>
-        </is>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Venda perdida (O produto não se encaixa à necessidade)</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>Funil Vendas Externas</t>
         </is>
       </c>
-      <c r="I3" s="0">
+      <c r="I7" s="1">
         <v>245000000</v>
       </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>30.03.2026 11:00:16</t>
-        </is>
-      </c>
-      <c r="K3" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="L3" s="0" t="inlineStr">
-        <is>
-          <t>08.04.2026 11:14:26</t>
-        </is>
-      </c>
-      <c r="M3" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="N3" s="0" t="inlineStr">
-        <is>
-          <t>Ricardo, Hermando Araujo</t>
-        </is>
-      </c>
-      <c r="P3" s="0" t="inlineStr">
-        <is>
-          <t>não fechado</t>
-        </is>
-      </c>
-      <c r="R3" s="0" t="inlineStr">
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>24.03.2026 17:42:10</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>08.04.2026 09:58:45</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>Koru Engenharia</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>Alexandre, Jordan imóveis</t>
+        </is>
+      </c>
+      <c r="P7" s="1" t="inlineStr">
+        <is>
+          <t>08.04.2026 09:58</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="inlineStr">
         <is>
           <t>Alameda dos ipês</t>
         </is>
       </c>
-      <c r="S3" s="0" t="inlineStr">
+      <c r="S7" s="1" t="inlineStr">
         <is>
           <t>Imobiliária</t>
         </is>
       </c>
-      <c r="AH3" s="0" t="inlineStr">
-        <is>
-          <t>85 997839573</t>
-        </is>
-      </c>
-      <c r="AN3" s="0" t="inlineStr">
-        <is>
-          <t>Carta de cancelamento</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" spans="1:40">
-      <c r="A4" s="0">
-        <v>36033076</v>
-      </c>
-      <c r="B4" s="0" t="inlineStr">
-        <is>
-          <t>Larissa</t>
-        </is>
-      </c>
-      <c r="F4" s="0" t="inlineStr">
-        <is>
-          <t>Comercial</t>
-        </is>
-      </c>
-      <c r="G4" s="0" t="inlineStr">
-        <is>
-          <t>Venda perdida (O produto não se encaixa à necessidade)</t>
-        </is>
-      </c>
-      <c r="H4" s="0" t="inlineStr">
-        <is>
-          <t>Funil Vendas Externas</t>
-        </is>
-      </c>
-      <c r="I4" s="0">
-        <v>245000000</v>
-      </c>
-      <c r="J4" s="0" t="inlineStr">
-        <is>
-          <t>24.03.2026 17:42:10</t>
-        </is>
-      </c>
-      <c r="K4" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="L4" s="0" t="inlineStr">
-        <is>
-          <t>08.04.2026 09:58:45</t>
-        </is>
-      </c>
-      <c r="M4" s="0" t="inlineStr">
-        <is>
-          <t>Koru Engenharia</t>
-        </is>
-      </c>
-      <c r="N4" s="0" t="inlineStr">
-        <is>
-          <t>Alexandre, Jordan imóveis</t>
-        </is>
-      </c>
-      <c r="P4" s="0" t="inlineStr">
-        <is>
-          <t>08.04.2026 09:58</t>
-        </is>
-      </c>
-      <c r="R4" s="0" t="inlineStr">
-        <is>
-          <t>Alameda dos ipês</t>
-        </is>
-      </c>
-      <c r="S4" s="0" t="inlineStr">
-        <is>
-          <t>Imobiliária</t>
-        </is>
-      </c>
-      <c r="AN4" s="0" t="inlineStr">
+      <c r="AO7" s="1" t="inlineStr">
         <is>
           <t>Falta imposto de renda</t>
         </is>

</xml_diff>